<commit_message>
Removed some unnecessary files
</commit_message>
<xml_diff>
--- a/src/test/resources/NegativeTestData.xlsx
+++ b/src/test/resources/NegativeTestData.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harsh\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Sprint\capgemini_Capstone_Project\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{387006A3-BE8F-4048-8534-0274581FCC51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFEE10D3-56BF-4C73-BA9E-B244C8CF3FA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FC2F7B09-4248-42F1-A7E5-E6ED8A97573C}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="48">
   <si>
     <t>TCID</t>
   </si>
@@ -99,9 +99,6 @@
     <t>expired_token_test_456</t>
   </si>
   <si>
-    <t>Wrong@Password02</t>
-  </si>
-  <si>
     <t>deleteFake002</t>
   </si>
   <si>
@@ -135,9 +132,6 @@
     <t>unauthorized_token_555</t>
   </si>
   <si>
-    <t>Incorrect123!</t>
-  </si>
-  <si>
     <t>deleteFake004</t>
   </si>
   <si>
@@ -153,9 +147,6 @@
     <t>invalid_jwt_token_demo</t>
   </si>
   <si>
-    <t>FakePassword@2026</t>
-  </si>
-  <si>
     <t>deleteFake005</t>
   </si>
   <si>
@@ -163,13 +154,37 @@
   </si>
   <si>
     <t>Login failure validation scenario</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>autoUser001@gmail.com</t>
+  </si>
+  <si>
+    <t>validuser@gmail.com</t>
+  </si>
+  <si>
+    <t>autoUser003@gmail.com</t>
+  </si>
+  <si>
+    <t>autoUser004@gmail.com</t>
+  </si>
+  <si>
+    <t>autoUSer005@gmail.com</t>
+  </si>
+  <si>
+    <t>Inco</t>
+  </si>
+  <si>
+    <t>FakePassword</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -181,6 +196,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -203,10 +226,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -214,8 +238,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -528,7 +559,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBC9C12D-4616-4497-ADFB-22C68B7DB47B}">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="34.77734375" customWidth="1"/>
@@ -540,30 +571,33 @@
     <col min="7" max="7" width="23.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
@@ -571,137 +605,160 @@
         <v>8</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="2">
+      <c r="E2" s="2">
         <v>0</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="72" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="2">
+      <c r="E3" s="2">
         <v>1.1111111111111099E+23</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="72" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2">
+        <v>2.2222222222222198E+23</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="2">
-        <v>2.2222222222222198E+23</v>
-      </c>
-      <c r="E4" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="G4" s="2" t="s">
+    </row>
+    <row r="5" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
         <v>24</v>
       </c>
+      <c r="B5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" s="2">
+        <v>3.3333333333333299E+23</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>29</v>
+      </c>
     </row>
-    <row r="5" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D5" s="2">
-        <v>3.3333333333333299E+23</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="G5" s="2" t="s">
+    <row r="6" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
         <v>30</v>
       </c>
+      <c r="B6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E6" s="2">
+        <v>4.4444444444444397E+23</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>34</v>
+      </c>
     </row>
-    <row r="6" spans="1:7" ht="72" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D6" s="2">
-        <v>4.4444444444444397E+23</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="F6" s="2" t="s">
+    <row r="7" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="B7" s="2" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" ht="72" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+      <c r="C7" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E7" s="2">
+        <v>5.5555555555555501E+23</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="G7" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="H7" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="D7" s="2">
-        <v>5.5555555555555501E+23</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>42</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C4" r:id="rId1" xr:uid="{12F98AFA-71ED-48B9-AE6A-82F3D5BA8620}"/>
+    <hyperlink ref="C5" r:id="rId2" xr:uid="{2DD309B8-229C-416F-BCCF-B88B28289192}"/>
+    <hyperlink ref="C6" r:id="rId3" xr:uid="{AD0AAAF9-774B-4BA3-89C1-BF0CCF3D02A9}"/>
+    <hyperlink ref="C7" r:id="rId4" xr:uid="{A41023BC-0688-4BF2-AB7B-0E0D4D49EB94}"/>
+    <hyperlink ref="C3" r:id="rId5" xr:uid="{B5EC5F6F-355B-477F-8B4B-37B4572583BD}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>